<commit_message>
fix: add expected column logic for valid vs invalid login tests
</commit_message>
<xml_diff>
--- a/testData/LoginData.xlsx
+++ b/testData/LoginData.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91797\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2E5F214-4D20-424B-AB32-A87405500E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2C5130-1DAA-4644-AC86-508713818F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
   <si>
     <t>Username</t>
   </si>
@@ -82,27 +82,15 @@
     <t>pass word</t>
   </si>
   <si>
-    <t>very_long_username_test_exceeding_standard_limits_999</t>
-  </si>
-  <si>
     <t>short</t>
   </si>
   <si>
-    <t>very_long_password_test_exceeding_standard_limits_999</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> OR '1'='1</t>
-  </si>
-  <si>
     <t>anything</t>
   </si>
   <si>
     <t>admin' --</t>
   </si>
   <si>
-    <t>&lt;script&gt;alert('xss')&lt;/script&gt;</t>
-  </si>
-  <si>
     <t>pass</t>
   </si>
   <si>
@@ -125,6 +113,21 @@
   </si>
   <si>
     <t>pass_03</t>
+  </si>
+  <si>
+    <t>Expected</t>
+  </si>
+  <si>
+    <t>very_long_username...</t>
+  </si>
+  <si>
+    <t>very_long...</t>
+  </si>
+  <si>
+    <t>OR '1'='1</t>
+  </si>
+  <si>
+    <t>script alert xss</t>
   </si>
 </sst>
 </file>
@@ -139,8 +142,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -167,8 +171,12 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -387,182 +395,243 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACB40DFA-CE15-4CDD-A893-CD15FDCFDEAC}">
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.6640625" customWidth="1"/>
+    <col min="1" max="1" width="16.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="C2" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="C3" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="C4" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="C5" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="C7" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="C8" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="C9" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="C10" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="C11" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="C14" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="C15" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C16" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>1234567890</v>
+      </c>
+      <c r="B17" s="2">
+        <v>987654321</v>
+      </c>
+      <c r="C17" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="B18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="B19" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C19" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>1234567890</v>
-      </c>
-      <c r="B17" s="1">
-        <v>987654321</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="C20" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B21" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>34</v>
+      <c r="C21" s="2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>